<commit_message>
update: curriculum lead correction, brand color rebrand, curriculum PDF
- Milestone 3 lead corrected to Mark + Cam (CFO) in curriculum.md and LSDE revision doc
- All 7 milestone Excel templates rebranded to approved black/gold palette
- Curriculum exported as clean formatted PDF (outputs/strategy/curriculum-business-without-you.pdf)
- Signature framework and funnel blueprint doc and PDF committed from prior session
</commit_message>
<xml_diff>
--- a/apps/bottleneck-breakthrough/Cool_Hollow_Coaching_Milestone_6_Bottleneck_Breakthrough_Template.xlsx
+++ b/apps/bottleneck-breakthrough/Cool_Hollow_Coaching_Milestone_6_Bottleneck_Breakthrough_Template.xlsx
@@ -35,17 +35,17 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="00E8C766"/>
       <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="000E4643"/>
+      <color rgb="001A1A1A"/>
       <sz val="12"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="000E4643"/>
+      <color rgb="001A1A1A"/>
       <sz val="11"/>
     </font>
     <font>
@@ -56,7 +56,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="000E4643"/>
+      <color rgb="001A1A1A"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -74,11 +74,11 @@
       <name val="Calibri"/>
       <b val="1"/>
       <i val="1"/>
-      <color rgb="000E4643"/>
+      <color rgb="001A1A1A"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -87,12 +87,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000E4643"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00589BA8"/>
+        <fgColor rgb="001A1A1A"/>
       </patternFill>
     </fill>
     <fill>
@@ -102,12 +97,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00B4D351"/>
+        <fgColor rgb="00E8C766"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FAF8F3"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -149,19 +144,19 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>

</xml_diff>